<commit_message>
DB1: regenerate playerDatabase.ts from SOT (Codex 5.5 build, Fable 5 audit: CONFORMS)
- 440 team players regenerated full-field from SOT workbook: ratings,
  positions/roles (Fenomeno corrected to SP/RP two-way, armSlot Sub),
  traits (13 normalizations), chemistry (CMP/CRA/DIS/SCH/SPI), arsenals
- armSlot added to schema: 179/179 pitchers (High 65/Mid 65/Low 44/Sub 5),
  never on hitters or free agents
- 66 free agents byte-identical; all player ids preserved
- F3 ruling: 4 SOT name typos fixed in workbook (Danno Yoshida, Seymour
  Socks, Lars Stadkleef, Pex Flexi per in-game check); regen rerun;
  explicit name map emptied
- Audit: independent extraction, 440/440 match, 18/18 ruling anchors,
  zero player-data-dependent test failures; 3 known baseline failures only
- Constants preview (V117 will commit): caps 1,323,633/1,169,013/1,048,489
- PROMPT_CONTRACTS: DB1-AUDIT contract; SESSION_LOG: build+audit+F3 record
</commit_message>
<xml_diff>
--- a/reference-docs/SOURCE_OF_TRUTH_Super Mega Baseball 4 Rosters.xlsx
+++ b/reference-docs/SOURCE_OF_TRUTH_Super Mega Baseball 4 Rosters.xlsx
@@ -3094,7 +3094,7 @@
       </c>
       <c r="B14" s="117" t="inlineStr">
         <is>
-          <t>Seymour Scoks</t>
+          <t>Seymour Socks</t>
         </is>
       </c>
       <c r="C14" s="117" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="B15" s="123" t="inlineStr">
         <is>
-          <t>Lars Stadkeleef</t>
+          <t>Lars Stadkleef</t>
         </is>
       </c>
       <c r="C15" s="123" t="inlineStr">
@@ -19473,7 +19473,7 @@
       </c>
       <c r="B11" s="259" t="inlineStr">
         <is>
-          <t>Pex Flext</t>
+          <t>Pex Flexi</t>
         </is>
       </c>
       <c r="C11" s="259" t="inlineStr">
@@ -31310,7 +31310,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Dano Yoshida</t>
+          <t>Danno Yoshida</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">

</xml_diff>